<commit_message>
Dodat automatski odabir K
</commit_message>
<xml_diff>
--- a/results/metrics/knn_izvjestaj.xlsx
+++ b/results/metrics/knn_izvjestaj.xlsx
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -534,7 +534,7 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>99.7%</t>
+          <t>99.1%</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -591,23 +591,6 @@
       <c r="C6" s="5" t="inlineStr">
         <is>
           <t>KNN hiperparametar</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Broj klasa</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>Low CLV, Mid CLV, High CLV</t>
         </is>
       </c>
     </row>
@@ -625,7 +608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -672,51 +655,51 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Mid CLV</t>
+          <t>Low CLV</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>0.9961</t>
+          <t>0.9930</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>1.0000</t>
+          <t>0.9972</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>0.9981</t>
+          <t>0.9951</t>
         </is>
       </c>
       <c r="E3" s="4" t="n">
-        <v>769</v>
+        <v>713</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>Low CLV</t>
+          <t>Very Low CLV</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>1.0000</t>
+          <t>0.9974</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>0.9925</t>
+          <t>0.9922</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>0.9963</t>
+          <t>0.9948</t>
         </is>
       </c>
       <c r="E4" s="6" t="n">
-        <v>402</v>
+        <v>386</v>
       </c>
     </row>
     <row r="5">
@@ -727,37 +710,87 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>1.0000</t>
+          <t>0.6000</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>1.0000</t>
+          <t>0.7500</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>1.0000</t>
+          <t>0.6667</t>
         </is>
       </c>
       <c r="E5" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Very High CLV</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Mid CLV</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>0.9577</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>0.9577</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>0.9577</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>Ukupna tačnost</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
-        <is>
-          <t>0.9974</t>
-        </is>
-      </c>
-      <c r="C6" s="9" t="inlineStr"/>
-      <c r="D6" s="9" t="inlineStr"/>
-      <c r="E6" s="9" t="n">
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>0.9906</t>
+        </is>
+      </c>
+      <c r="C8" s="9" t="inlineStr"/>
+      <c r="D8" s="9" t="inlineStr"/>
+      <c r="E8" s="9" t="n">
         <v>1176</v>
       </c>
     </row>
@@ -775,7 +808,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -799,50 +832,72 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
+          <t>Low CLV</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Very Low CLV</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>High CLV</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Very High CLV</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
           <t>Mid CLV</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Low CLV</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>High CLV</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Mid CLV</t>
+          <t>Low CLV</t>
         </is>
       </c>
       <c r="B3" s="9" t="n">
-        <v>769</v>
-      </c>
-      <c r="C3" s="4" t="n">
-        <v>0</v>
+        <v>711</v>
+      </c>
+      <c r="C3" s="11" t="n">
+        <v>1</v>
       </c>
       <c r="D3" s="4" t="n">
         <v>0</v>
+      </c>
+      <c r="E3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="11" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Low CLV</t>
+          <t>Very Low CLV</t>
         </is>
       </c>
       <c r="B4" s="11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C4" s="9" t="n">
-        <v>399</v>
+        <v>383</v>
       </c>
       <c r="D4" s="4" t="n">
         <v>0</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="11" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -858,7 +913,57 @@
         <v>0</v>
       </c>
       <c r="D5" s="9" t="n">
-        <v>5</v>
+        <v>3</v>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Very High CLV</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Mid CLV</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="9" t="n">
+        <v>68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
6 klastera, za KNN pravim Low, Mid, High
</commit_message>
<xml_diff>
--- a/results/metrics/knn_izvjestaj.xlsx
+++ b/results/metrics/knn_izvjestaj.xlsx
@@ -534,7 +534,7 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>99.1%</t>
+          <t>99.5%</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -608,7 +608,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -653,144 +653,155 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Low CLV</t>
-        </is>
+      <c r="A3" s="3" t="n">
+        <v>0</v>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>0.9930</t>
+          <t>0.9974</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
+          <t>0.9948</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>0.9961</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="n">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>0.9959</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>0.9986</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
           <t>0.9972</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>0.9951</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="n">
-        <v>713</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>Very Low CLV</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>0.9974</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>0.9922</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>0.9948</t>
-        </is>
-      </c>
       <c r="E4" s="6" t="n">
-        <v>386</v>
+        <v>723</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>High CLV</t>
-        </is>
+      <c r="A5" s="3" t="n">
+        <v>2</v>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>0.6000</t>
+          <t>0.0000</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>0.0000</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>0.9839</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>0.9839</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>0.9839</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
           <t>0.7500</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>0.6667</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="n">
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>0.7500</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>0.7500</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>Very High CLV</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>0.0000</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>0.0000</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>0.0000</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Mid CLV</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>0.9577</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>0.9577</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>0.9577</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="n">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>Ukupna tačnost</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>0.9906</t>
-        </is>
-      </c>
-      <c r="C8" s="9" t="inlineStr"/>
-      <c r="D8" s="9" t="inlineStr"/>
-      <c r="E8" s="9" t="n">
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>0.9949</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="n">
         <v>1176</v>
       </c>
     </row>
@@ -808,13 +819,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="25" customHeight="1">
@@ -830,140 +844,161 @@
           <t>Stvarno \ Predviđeno</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Low CLV</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Very Low CLV</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>High CLV</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Very High CLV</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Mid CLV</t>
-        </is>
+      <c r="B2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Low CLV</t>
-        </is>
+      <c r="A3" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="B3" s="9" t="n">
-        <v>711</v>
+        <v>384</v>
       </c>
       <c r="C3" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" s="11" t="n">
+      <c r="B4" s="11" t="n">
         <v>1</v>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Very Low CLV</t>
-        </is>
-      </c>
-      <c r="B4" s="11" t="n">
+      <c r="C4" s="9" t="n">
+        <v>722</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="C4" s="9" t="n">
-        <v>383</v>
-      </c>
-      <c r="D4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="11" t="n">
+      <c r="B5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="11" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>High CLV</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D5" s="9" t="n">
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="9" t="n">
+        <v>61</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="9" t="n">
         <v>3</v>
-      </c>
-      <c r="E5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" s="11" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Very High CLV</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="E6" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" s="4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Mid CLV</t>
-        </is>
-      </c>
-      <c r="B7" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="C7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" s="9" t="n">
-        <v>68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>